<commit_message>
Update extract historical vul Melhoria de performance.
</commit_message>
<xml_diff>
--- a/resources/annotated_java_vulnerabilities.xlsx
+++ b/resources/annotated_java_vulnerabilities.xlsx
@@ -34,7 +34,7 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mg8wg0lPQ89D2o7W8G7KezR+v0STA=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mhRlG5RYnavp99VoIBycUoHdky9OA=="/>
     </ext>
   </extLst>
 </comments>
@@ -5607,7 +5607,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="1">
       <c r="A2" s="3" t="s">
         <v>23</v>
       </c>
@@ -5745,7 +5745,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="1">
       <c r="A4" s="3" t="s">
         <v>33</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="1">
       <c r="A5" s="3" t="s">
         <v>38</v>
       </c>
@@ -5889,7 +5889,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="1">
       <c r="A6" s="3" t="s">
         <v>43</v>
       </c>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="W6" s="7"/>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" s="3" t="s">
         <v>46</v>
       </c>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="W7" s="7"/>
     </row>
-    <row r="8">
+    <row r="8" hidden="1">
       <c r="A8" s="3" t="s">
         <v>49</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="1">
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
@@ -6169,7 +6169,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
@@ -6377,7 +6377,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="1">
       <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
@@ -6445,7 +6445,7 @@
       </c>
       <c r="W13" s="7"/>
     </row>
-    <row r="14">
+    <row r="14" hidden="1">
       <c r="A14" s="3" t="s">
         <v>67</v>
       </c>
@@ -6587,7 +6587,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="1">
       <c r="A16" s="3" t="s">
         <v>73</v>
       </c>
@@ -6659,7 +6659,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" s="3" t="s">
         <v>77</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="1">
       <c r="A18" s="3" t="s">
         <v>82</v>
       </c>
@@ -6803,7 +6803,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="1">
       <c r="A19" s="3" t="s">
         <v>85</v>
       </c>
@@ -6875,7 +6875,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="1">
       <c r="A20" s="3" t="s">
         <v>89</v>
       </c>
@@ -6947,7 +6947,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="1">
       <c r="A21" s="3" t="s">
         <v>93</v>
       </c>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="W21" s="7"/>
     </row>
-    <row r="22">
+    <row r="22" hidden="1">
       <c r="A22" s="3" t="s">
         <v>95</v>
       </c>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="W22" s="7"/>
     </row>
-    <row r="23">
+    <row r="23" hidden="1">
       <c r="A23" s="3" t="s">
         <v>97</v>
       </c>
@@ -7155,7 +7155,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="1">
       <c r="A24" s="3" t="s">
         <v>101</v>
       </c>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="W24" s="7"/>
     </row>
-    <row r="25">
+    <row r="25" hidden="1">
       <c r="A25" s="3" t="s">
         <v>104</v>
       </c>
@@ -7295,7 +7295,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="1">
       <c r="A26" s="3" t="s">
         <v>107</v>
       </c>
@@ -7367,7 +7367,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="1">
       <c r="A27" s="3" t="s">
         <v>110</v>
       </c>
@@ -7439,7 +7439,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="1">
       <c r="A28" s="3" t="s">
         <v>113</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="1">
       <c r="A30" s="3" t="s">
         <v>116</v>
       </c>
@@ -7653,7 +7653,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="1">
       <c r="A31" s="3" t="s">
         <v>116</v>
       </c>
@@ -7725,7 +7725,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="1">
       <c r="A32" s="3" t="s">
         <v>116</v>
       </c>
@@ -7797,7 +7797,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="1">
       <c r="A33" s="3" t="s">
         <v>116</v>
       </c>
@@ -7939,7 +7939,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="1">
       <c r="A35" s="3" t="s">
         <v>116</v>
       </c>
@@ -8011,7 +8011,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="1">
       <c r="A36" s="3" t="s">
         <v>116</v>
       </c>
@@ -8083,7 +8083,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="1">
       <c r="A37" s="3" t="s">
         <v>116</v>
       </c>
@@ -8225,7 +8225,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="1">
       <c r="A39" s="3" t="s">
         <v>116</v>
       </c>
@@ -8297,7 +8297,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="1">
       <c r="A40" s="3" t="s">
         <v>116</v>
       </c>
@@ -8369,7 +8369,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="1">
       <c r="A41" s="3" t="s">
         <v>116</v>
       </c>
@@ -8441,7 +8441,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="1">
       <c r="A42" s="3" t="s">
         <v>116</v>
       </c>
@@ -8513,7 +8513,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" hidden="1">
       <c r="A43" s="3" t="s">
         <v>116</v>
       </c>
@@ -8585,7 +8585,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" hidden="1">
       <c r="A44" s="3" t="s">
         <v>116</v>
       </c>
@@ -8657,7 +8657,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="1">
       <c r="A45" s="3" t="s">
         <v>116</v>
       </c>
@@ -8725,7 +8725,7 @@
       </c>
       <c r="W45" s="7"/>
     </row>
-    <row r="46">
+    <row r="46" hidden="1">
       <c r="A46" s="3" t="s">
         <v>116</v>
       </c>
@@ -8797,7 +8797,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" hidden="1">
       <c r="A47" s="3" t="s">
         <v>116</v>
       </c>
@@ -8869,7 +8869,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="1">
       <c r="A48" s="3" t="s">
         <v>116</v>
       </c>
@@ -9011,7 +9011,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" hidden="1">
       <c r="A50" s="3" t="s">
         <v>116</v>
       </c>
@@ -9083,7 +9083,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" hidden="1">
       <c r="A51" s="3" t="s">
         <v>116</v>
       </c>
@@ -9151,7 +9151,7 @@
       </c>
       <c r="W51" s="7"/>
     </row>
-    <row r="52">
+    <row r="52" hidden="1">
       <c r="A52" s="3" t="s">
         <v>116</v>
       </c>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="W52" s="7"/>
     </row>
-    <row r="53">
+    <row r="53" hidden="1">
       <c r="A53" s="3" t="s">
         <v>116</v>
       </c>
@@ -9291,7 +9291,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" hidden="1">
       <c r="A54" s="3" t="s">
         <v>116</v>
       </c>
@@ -9499,7 +9499,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" hidden="1">
       <c r="A57" s="3" t="s">
         <v>116</v>
       </c>
@@ -9641,7 +9641,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" hidden="1">
       <c r="A59" s="3" t="s">
         <v>116</v>
       </c>
@@ -9713,7 +9713,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" hidden="1">
       <c r="A60" s="3" t="s">
         <v>116</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" hidden="1">
       <c r="A61" s="3" t="s">
         <v>116</v>
       </c>
@@ -9927,7 +9927,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" hidden="1">
       <c r="A63" s="3" t="s">
         <v>116</v>
       </c>
@@ -9999,7 +9999,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" hidden="1">
       <c r="A64" s="3" t="s">
         <v>116</v>
       </c>
@@ -10071,7 +10071,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" hidden="1">
       <c r="A65" s="3" t="s">
         <v>116</v>
       </c>
@@ -10143,7 +10143,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" hidden="1">
       <c r="A66" s="3" t="s">
         <v>116</v>
       </c>
@@ -10215,7 +10215,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" hidden="1">
       <c r="A67" s="3" t="s">
         <v>116</v>
       </c>
@@ -10287,7 +10287,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" hidden="1">
       <c r="A68" s="3" t="s">
         <v>116</v>
       </c>
@@ -10359,7 +10359,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" hidden="1">
       <c r="A69" s="3" t="s">
         <v>116</v>
       </c>
@@ -10501,7 +10501,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" hidden="1">
       <c r="A71" s="3" t="s">
         <v>116</v>
       </c>
@@ -10573,7 +10573,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" hidden="1">
       <c r="A72" s="3" t="s">
         <v>116</v>
       </c>
@@ -10645,7 +10645,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" hidden="1">
       <c r="A73" s="3" t="s">
         <v>116</v>
       </c>
@@ -10717,7 +10717,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" hidden="1">
       <c r="A74" s="3" t="s">
         <v>116</v>
       </c>
@@ -10789,7 +10789,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" hidden="1">
       <c r="A75" s="3" t="s">
         <v>116</v>
       </c>
@@ -10861,7 +10861,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" hidden="1">
       <c r="A76" s="3" t="s">
         <v>116</v>
       </c>
@@ -10933,7 +10933,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" hidden="1">
       <c r="A77" s="3" t="s">
         <v>116</v>
       </c>
@@ -11071,7 +11071,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" hidden="1">
       <c r="A79" s="3" t="s">
         <v>116</v>
       </c>
@@ -11143,7 +11143,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" hidden="1">
       <c r="A80" s="3" t="s">
         <v>116</v>
       </c>
@@ -11215,7 +11215,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" hidden="1">
       <c r="A81" s="3" t="s">
         <v>116</v>
       </c>
@@ -11287,7 +11287,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" hidden="1">
       <c r="A82" s="3" t="s">
         <v>116</v>
       </c>
@@ -11359,7 +11359,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" hidden="1">
       <c r="A83" s="3" t="s">
         <v>116</v>
       </c>
@@ -11431,7 +11431,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" hidden="1">
       <c r="A84" s="3" t="s">
         <v>116</v>
       </c>
@@ -11503,7 +11503,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" hidden="1">
       <c r="A85" s="3" t="s">
         <v>116</v>
       </c>
@@ -11571,7 +11571,7 @@
       </c>
       <c r="W85" s="7"/>
     </row>
-    <row r="86">
+    <row r="86" hidden="1">
       <c r="A86" s="3" t="s">
         <v>116</v>
       </c>
@@ -11639,7 +11639,7 @@
       </c>
       <c r="W86" s="7"/>
     </row>
-    <row r="87">
+    <row r="87" hidden="1">
       <c r="A87" s="3" t="s">
         <v>116</v>
       </c>
@@ -11707,7 +11707,7 @@
       </c>
       <c r="W87" s="7"/>
     </row>
-    <row r="88">
+    <row r="88" hidden="1">
       <c r="A88" s="3" t="s">
         <v>116</v>
       </c>
@@ -11849,7 +11849,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" hidden="1">
       <c r="A90" s="3" t="s">
         <v>245</v>
       </c>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="W90" s="7"/>
     </row>
-    <row r="91">
+    <row r="91" hidden="1">
       <c r="A91" s="3" t="s">
         <v>248</v>
       </c>
@@ -12059,7 +12059,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" hidden="1">
       <c r="A93" s="3" t="s">
         <v>254</v>
       </c>
@@ -12127,7 +12127,7 @@
       </c>
       <c r="W93" s="7"/>
     </row>
-    <row r="94">
+    <row r="94" hidden="1">
       <c r="A94" s="3" t="s">
         <v>257</v>
       </c>
@@ -12199,7 +12199,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" hidden="1">
       <c r="A95" s="3" t="s">
         <v>261</v>
       </c>
@@ -12341,7 +12341,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" hidden="1">
       <c r="A97" s="3" t="s">
         <v>268</v>
       </c>
@@ -12413,7 +12413,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" hidden="1">
       <c r="A98" s="3" t="s">
         <v>271</v>
       </c>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="W98" s="7"/>
     </row>
-    <row r="99">
+    <row r="99" hidden="1">
       <c r="A99" s="3" t="s">
         <v>273</v>
       </c>
@@ -12623,7 +12623,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" hidden="1">
       <c r="A101" s="3" t="s">
         <v>277</v>
       </c>
@@ -12695,7 +12695,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" hidden="1">
       <c r="A102" s="3" t="s">
         <v>282</v>
       </c>
@@ -12763,7 +12763,7 @@
       </c>
       <c r="W102" s="7"/>
     </row>
-    <row r="103">
+    <row r="103" hidden="1">
       <c r="A103" s="3" t="s">
         <v>285</v>
       </c>
@@ -12905,7 +12905,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" hidden="1">
       <c r="A105" s="3" t="s">
         <v>290</v>
       </c>
@@ -12977,7 +12977,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" hidden="1">
       <c r="A106" s="3" t="s">
         <v>292</v>
       </c>
@@ -13045,7 +13045,7 @@
       </c>
       <c r="W106" s="7"/>
     </row>
-    <row r="107">
+    <row r="107" hidden="1">
       <c r="A107" s="3" t="s">
         <v>292</v>
       </c>
@@ -13113,7 +13113,7 @@
       </c>
       <c r="W107" s="7"/>
     </row>
-    <row r="108">
+    <row r="108" hidden="1">
       <c r="A108" s="3" t="s">
         <v>298</v>
       </c>
@@ -13181,7 +13181,7 @@
       </c>
       <c r="W108" s="7"/>
     </row>
-    <row r="109">
+    <row r="109" hidden="1">
       <c r="A109" s="3" t="s">
         <v>301</v>
       </c>
@@ -13249,7 +13249,7 @@
       </c>
       <c r="W109" s="7"/>
     </row>
-    <row r="110">
+    <row r="110" hidden="1">
       <c r="A110" s="3" t="s">
         <v>305</v>
       </c>
@@ -13321,7 +13321,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" hidden="1">
       <c r="A111" s="3" t="s">
         <v>308</v>
       </c>
@@ -13393,7 +13393,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" hidden="1">
       <c r="A112" s="3" t="s">
         <v>311</v>
       </c>
@@ -13465,7 +13465,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" hidden="1">
       <c r="A113" s="3" t="s">
         <v>314</v>
       </c>
@@ -13533,7 +13533,7 @@
       </c>
       <c r="W113" s="7"/>
     </row>
-    <row r="114">
+    <row r="114" hidden="1">
       <c r="A114" s="3" t="s">
         <v>316</v>
       </c>
@@ -13605,7 +13605,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" hidden="1">
       <c r="A115" s="3" t="s">
         <v>320</v>
       </c>
@@ -13677,7 +13677,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" hidden="1">
       <c r="A116" s="3" t="s">
         <v>322</v>
       </c>
@@ -13749,7 +13749,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" hidden="1">
       <c r="A117" s="3" t="s">
         <v>324</v>
       </c>
@@ -13821,7 +13821,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" hidden="1">
       <c r="A118" s="3" t="s">
         <v>327</v>
       </c>
@@ -13889,7 +13889,7 @@
       </c>
       <c r="W118" s="7"/>
     </row>
-    <row r="119">
+    <row r="119" hidden="1">
       <c r="A119" s="3" t="s">
         <v>330</v>
       </c>
@@ -14031,7 +14031,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" hidden="1">
       <c r="A121" s="3" t="s">
         <v>335</v>
       </c>
@@ -14169,7 +14169,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" hidden="1">
       <c r="A123" s="3" t="s">
         <v>341</v>
       </c>
@@ -14241,7 +14241,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" hidden="1">
       <c r="A124" s="3" t="s">
         <v>344</v>
       </c>
@@ -14383,7 +14383,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" hidden="1">
       <c r="A126" s="3" t="s">
         <v>349</v>
       </c>
@@ -14455,7 +14455,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" hidden="1">
       <c r="A127" s="3" t="s">
         <v>352</v>
       </c>
@@ -14527,7 +14527,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" hidden="1">
       <c r="A128" s="3" t="s">
         <v>356</v>
       </c>
@@ -14599,7 +14599,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" hidden="1">
       <c r="A129" s="3" t="s">
         <v>357</v>
       </c>
@@ -14671,7 +14671,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" hidden="1">
       <c r="A130" s="3" t="s">
         <v>359</v>
       </c>
@@ -14743,7 +14743,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" hidden="1">
       <c r="A131" s="3" t="s">
         <v>362</v>
       </c>
@@ -14815,7 +14815,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" hidden="1">
       <c r="A132" s="3" t="s">
         <v>365</v>
       </c>
@@ -14887,7 +14887,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" hidden="1">
       <c r="A133" s="3" t="s">
         <v>368</v>
       </c>
@@ -14959,7 +14959,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" hidden="1">
       <c r="A134" s="3" t="s">
         <v>371</v>
       </c>
@@ -15031,7 +15031,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" hidden="1">
       <c r="A135" s="3" t="s">
         <v>374</v>
       </c>
@@ -15103,7 +15103,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" hidden="1">
       <c r="A136" s="3" t="s">
         <v>377</v>
       </c>
@@ -15171,7 +15171,7 @@
       </c>
       <c r="W136" s="7"/>
     </row>
-    <row r="137">
+    <row r="137" hidden="1">
       <c r="A137" s="3" t="s">
         <v>380</v>
       </c>
@@ -15243,7 +15243,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" hidden="1">
       <c r="A138" s="3" t="s">
         <v>383</v>
       </c>
@@ -15385,7 +15385,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" hidden="1">
       <c r="A140" s="3" t="s">
         <v>387</v>
       </c>
@@ -15457,7 +15457,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" hidden="1">
       <c r="A141" s="3" t="s">
         <v>390</v>
       </c>
@@ -15529,7 +15529,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" hidden="1">
       <c r="A142" s="3" t="s">
         <v>393</v>
       </c>
@@ -15599,7 +15599,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" hidden="1">
       <c r="A143" s="3" t="s">
         <v>396</v>
       </c>
@@ -15671,7 +15671,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" hidden="1">
       <c r="A144" s="3" t="s">
         <v>399</v>
       </c>
@@ -15743,7 +15743,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" hidden="1">
       <c r="A145" s="3" t="s">
         <v>401</v>
       </c>
@@ -15815,7 +15815,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" hidden="1">
       <c r="A146" s="3" t="s">
         <v>403</v>
       </c>
@@ -15887,7 +15887,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" hidden="1">
       <c r="A147" s="3" t="s">
         <v>406</v>
       </c>
@@ -15959,7 +15959,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" hidden="1">
       <c r="A148" s="3" t="s">
         <v>409</v>
       </c>
@@ -16031,7 +16031,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" hidden="1">
       <c r="A149" s="3" t="s">
         <v>412</v>
       </c>
@@ -16103,7 +16103,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" hidden="1">
       <c r="A150" s="3" t="s">
         <v>415</v>
       </c>
@@ -16175,7 +16175,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" hidden="1">
       <c r="A151" s="3" t="s">
         <v>418</v>
       </c>
@@ -16247,7 +16247,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" hidden="1">
       <c r="A152" s="3" t="s">
         <v>418</v>
       </c>
@@ -16315,7 +16315,7 @@
       </c>
       <c r="W152" s="7"/>
     </row>
-    <row r="153" ht="15.75" customHeight="1">
+    <row r="153" ht="15.75" hidden="1" customHeight="1">
       <c r="A153" s="3" t="s">
         <v>418</v>
       </c>
@@ -16457,7 +16457,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" hidden="1">
       <c r="A155" s="3" t="s">
         <v>427</v>
       </c>
@@ -16529,7 +16529,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" hidden="1">
       <c r="A156" s="3" t="s">
         <v>429</v>
       </c>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="W156" s="7"/>
     </row>
-    <row r="157">
+    <row r="157" hidden="1">
       <c r="A157" s="3" t="s">
         <v>432</v>
       </c>
@@ -16669,7 +16669,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" hidden="1">
       <c r="A158" s="3" t="s">
         <v>434</v>
       </c>
@@ -16741,7 +16741,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" hidden="1">
       <c r="A159" s="3" t="s">
         <v>437</v>
       </c>
@@ -16813,7 +16813,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" hidden="1">
       <c r="A160" s="3" t="s">
         <v>440</v>
       </c>
@@ -16885,7 +16885,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" hidden="1">
       <c r="A161" s="3" t="s">
         <v>440</v>
       </c>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="W161" s="7"/>
     </row>
-    <row r="162">
+    <row r="162" hidden="1">
       <c r="A162" s="3" t="s">
         <v>445</v>
       </c>
@@ -17095,7 +17095,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" hidden="1">
       <c r="A164" s="3" t="s">
         <v>451</v>
       </c>
@@ -17163,7 +17163,7 @@
       </c>
       <c r="W164" s="7"/>
     </row>
-    <row r="165">
+    <row r="165" hidden="1">
       <c r="A165" s="3" t="s">
         <v>454</v>
       </c>
@@ -17231,7 +17231,7 @@
       </c>
       <c r="W165" s="7"/>
     </row>
-    <row r="166">
+    <row r="166" hidden="1">
       <c r="A166" s="3" t="s">
         <v>457</v>
       </c>
@@ -17373,7 +17373,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" hidden="1">
       <c r="A168" s="3" t="s">
         <v>462</v>
       </c>
@@ -17445,7 +17445,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" hidden="1">
       <c r="A169" s="3" t="s">
         <v>464</v>
       </c>
@@ -17517,7 +17517,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" hidden="1">
       <c r="A170" s="3" t="s">
         <v>467</v>
       </c>
@@ -17585,7 +17585,7 @@
       </c>
       <c r="W170" s="7"/>
     </row>
-    <row r="171">
+    <row r="171" hidden="1">
       <c r="A171" s="3" t="s">
         <v>470</v>
       </c>
@@ -17657,7 +17657,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" hidden="1">
       <c r="A172" s="3" t="s">
         <v>473</v>
       </c>
@@ -17729,7 +17729,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" hidden="1">
       <c r="A173" s="3" t="s">
         <v>475</v>
       </c>
@@ -17797,7 +17797,7 @@
       </c>
       <c r="W173" s="7"/>
     </row>
-    <row r="174">
+    <row r="174" hidden="1">
       <c r="A174" s="3" t="s">
         <v>478</v>
       </c>
@@ -17869,7 +17869,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" hidden="1">
       <c r="A175" s="3" t="s">
         <v>481</v>
       </c>
@@ -17941,7 +17941,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" hidden="1">
       <c r="A176" s="3" t="s">
         <v>484</v>
       </c>
@@ -18013,7 +18013,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" hidden="1">
       <c r="A177" s="3" t="s">
         <v>487</v>
       </c>
@@ -18085,7 +18085,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" hidden="1">
       <c r="A178" s="3" t="s">
         <v>490</v>
       </c>
@@ -18157,7 +18157,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" hidden="1">
       <c r="A179" s="3" t="s">
         <v>490</v>
       </c>
@@ -18229,7 +18229,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" hidden="1">
       <c r="A180" s="3" t="s">
         <v>494</v>
       </c>
@@ -18297,7 +18297,7 @@
       </c>
       <c r="W180" s="7"/>
     </row>
-    <row r="181">
+    <row r="181" hidden="1">
       <c r="A181" s="3" t="s">
         <v>494</v>
       </c>
@@ -18365,7 +18365,7 @@
       </c>
       <c r="W181" s="7"/>
     </row>
-    <row r="182">
+    <row r="182" hidden="1">
       <c r="A182" s="3" t="s">
         <v>499</v>
       </c>
@@ -18507,7 +18507,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" hidden="1">
       <c r="A184" s="3" t="s">
         <v>505</v>
       </c>
@@ -18579,7 +18579,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="185">
+    <row r="185" hidden="1">
       <c r="A185" s="3" t="s">
         <v>505</v>
       </c>
@@ -18651,7 +18651,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="186">
+    <row r="186" hidden="1">
       <c r="A186" s="3" t="s">
         <v>505</v>
       </c>
@@ -18719,7 +18719,7 @@
       </c>
       <c r="W186" s="7"/>
     </row>
-    <row r="187">
+    <row r="187" hidden="1">
       <c r="A187" s="3" t="s">
         <v>505</v>
       </c>
@@ -18861,7 +18861,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="189">
+    <row r="189" hidden="1">
       <c r="A189" s="3" t="s">
         <v>517</v>
       </c>
@@ -18933,7 +18933,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="190">
+    <row r="190" hidden="1">
       <c r="A190" s="3" t="s">
         <v>520</v>
       </c>
@@ -19005,7 +19005,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="191">
+    <row r="191" hidden="1">
       <c r="A191" s="3" t="s">
         <v>520</v>
       </c>
@@ -19077,7 +19077,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="192">
+    <row r="192" hidden="1">
       <c r="A192" s="3" t="s">
         <v>525</v>
       </c>
@@ -19149,7 +19149,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="193">
+    <row r="193" hidden="1">
       <c r="A193" s="3" t="s">
         <v>528</v>
       </c>
@@ -19221,7 +19221,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="194">
+    <row r="194" hidden="1">
       <c r="A194" s="3" t="s">
         <v>530</v>
       </c>
@@ -19293,7 +19293,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="195">
+    <row r="195" hidden="1">
       <c r="A195" s="3" t="s">
         <v>533</v>
       </c>
@@ -19365,7 +19365,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="196">
+    <row r="196" hidden="1">
       <c r="A196" s="3" t="s">
         <v>536</v>
       </c>
@@ -19437,7 +19437,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="197">
+    <row r="197" hidden="1">
       <c r="A197" s="3" t="s">
         <v>539</v>
       </c>
@@ -19505,7 +19505,7 @@
       </c>
       <c r="W197" s="7"/>
     </row>
-    <row r="198">
+    <row r="198" hidden="1">
       <c r="A198" s="3" t="s">
         <v>543</v>
       </c>
@@ -19643,7 +19643,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="200">
+    <row r="200" hidden="1">
       <c r="A200" s="3" t="s">
         <v>546</v>
       </c>
@@ -19715,7 +19715,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="201">
+    <row r="201" hidden="1">
       <c r="A201" s="3" t="s">
         <v>551</v>
       </c>
@@ -19783,7 +19783,7 @@
       </c>
       <c r="W201" s="7"/>
     </row>
-    <row r="202">
+    <row r="202" hidden="1">
       <c r="A202" s="3" t="s">
         <v>551</v>
       </c>
@@ -19855,7 +19855,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="203">
+    <row r="203" hidden="1">
       <c r="A203" s="3" t="s">
         <v>551</v>
       </c>
@@ -19927,7 +19927,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="204">
+    <row r="204" hidden="1">
       <c r="A204" s="3" t="s">
         <v>551</v>
       </c>
@@ -19995,7 +19995,7 @@
       </c>
       <c r="W204" s="7"/>
     </row>
-    <row r="205">
+    <row r="205" hidden="1">
       <c r="A205" s="3" t="s">
         <v>560</v>
       </c>
@@ -20137,7 +20137,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="207">
+    <row r="207" hidden="1">
       <c r="A207" s="3" t="s">
         <v>565</v>
       </c>
@@ -20209,7 +20209,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="208">
+    <row r="208" hidden="1">
       <c r="A208" s="3" t="s">
         <v>568</v>
       </c>
@@ -20277,7 +20277,7 @@
       </c>
       <c r="W208" s="7"/>
     </row>
-    <row r="209">
+    <row r="209" hidden="1">
       <c r="A209" s="3" t="s">
         <v>571</v>
       </c>
@@ -20349,7 +20349,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="210">
+    <row r="210" hidden="1">
       <c r="A210" s="3" t="s">
         <v>573</v>
       </c>
@@ -20421,7 +20421,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="211">
+    <row r="211" hidden="1">
       <c r="A211" s="3" t="s">
         <v>573</v>
       </c>
@@ -20493,7 +20493,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="212">
+    <row r="212" hidden="1">
       <c r="A212" s="3" t="s">
         <v>578</v>
       </c>
@@ -20565,7 +20565,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="213">
+    <row r="213" hidden="1">
       <c r="A213" s="3" t="s">
         <v>582</v>
       </c>
@@ -20637,7 +20637,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="214">
+    <row r="214" hidden="1">
       <c r="A214" s="3" t="s">
         <v>585</v>
       </c>
@@ -20709,7 +20709,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="215">
+    <row r="215" hidden="1">
       <c r="A215" s="3" t="s">
         <v>588</v>
       </c>
@@ -20851,7 +20851,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="217">
+    <row r="217" hidden="1">
       <c r="A217" s="3" t="s">
         <v>593</v>
       </c>
@@ -20923,7 +20923,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="218">
+    <row r="218" hidden="1">
       <c r="A218" s="3" t="s">
         <v>593</v>
       </c>
@@ -20995,7 +20995,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="219">
+    <row r="219" hidden="1">
       <c r="A219" s="3" t="s">
         <v>593</v>
       </c>
@@ -21067,7 +21067,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="220">
+    <row r="220" hidden="1">
       <c r="A220" s="3" t="s">
         <v>593</v>
       </c>
@@ -21139,7 +21139,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="221">
+    <row r="221" hidden="1">
       <c r="A221" s="3" t="s">
         <v>602</v>
       </c>
@@ -21207,7 +21207,7 @@
       </c>
       <c r="W221" s="7"/>
     </row>
-    <row r="222">
+    <row r="222" hidden="1">
       <c r="A222" s="3" t="s">
         <v>605</v>
       </c>
@@ -21275,7 +21275,7 @@
       </c>
       <c r="W222" s="7"/>
     </row>
-    <row r="223">
+    <row r="223" hidden="1">
       <c r="A223" s="3" t="s">
         <v>608</v>
       </c>
@@ -21347,7 +21347,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="224">
+    <row r="224" hidden="1">
       <c r="A224" s="3" t="s">
         <v>610</v>
       </c>
@@ -21419,7 +21419,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="225">
+    <row r="225" hidden="1">
       <c r="A225" s="3" t="s">
         <v>613</v>
       </c>
@@ -21491,7 +21491,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="226">
+    <row r="226" hidden="1">
       <c r="A226" s="3" t="s">
         <v>616</v>
       </c>
@@ -21559,7 +21559,7 @@
       </c>
       <c r="W226" s="7"/>
     </row>
-    <row r="227">
+    <row r="227" hidden="1">
       <c r="A227" s="3" t="s">
         <v>619</v>
       </c>
@@ -21631,7 +21631,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="228">
+    <row r="228" hidden="1">
       <c r="A228" s="15" t="s">
         <v>622</v>
       </c>
@@ -21773,7 +21773,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="230">
+    <row r="230" hidden="1">
       <c r="A230" s="3" t="s">
         <v>626</v>
       </c>
@@ -21845,7 +21845,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="231">
+    <row r="231" hidden="1">
       <c r="A231" s="3" t="s">
         <v>628</v>
       </c>
@@ -21917,7 +21917,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" hidden="1">
       <c r="A232" s="3" t="s">
         <v>631</v>
       </c>
@@ -21989,7 +21989,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="233">
+    <row r="233" hidden="1">
       <c r="A233" s="3" t="s">
         <v>634</v>
       </c>
@@ -22061,7 +22061,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="234">
+    <row r="234" hidden="1">
       <c r="A234" s="3" t="s">
         <v>636</v>
       </c>
@@ -22133,7 +22133,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="235">
+    <row r="235" hidden="1">
       <c r="A235" s="3" t="s">
         <v>639</v>
       </c>
@@ -22201,7 +22201,7 @@
       </c>
       <c r="W235" s="7"/>
     </row>
-    <row r="236">
+    <row r="236" hidden="1">
       <c r="A236" s="3" t="s">
         <v>642</v>
       </c>
@@ -22273,7 +22273,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="237">
+    <row r="237" hidden="1">
       <c r="A237" s="3" t="s">
         <v>644</v>
       </c>
@@ -22345,7 +22345,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="238">
+    <row r="238" hidden="1">
       <c r="A238" s="3" t="s">
         <v>644</v>
       </c>
@@ -22417,7 +22417,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="239">
+    <row r="239" hidden="1">
       <c r="A239" s="3" t="s">
         <v>644</v>
       </c>
@@ -22489,7 +22489,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="240">
+    <row r="240" hidden="1">
       <c r="A240" s="3" t="s">
         <v>644</v>
       </c>
@@ -22561,7 +22561,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="241">
+    <row r="241" hidden="1">
       <c r="A241" s="3" t="s">
         <v>644</v>
       </c>
@@ -22699,7 +22699,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="243">
+    <row r="243" hidden="1">
       <c r="A243" s="3" t="s">
         <v>644</v>
       </c>
@@ -22769,7 +22769,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="244">
+    <row r="244" hidden="1">
       <c r="A244" s="3" t="s">
         <v>644</v>
       </c>
@@ -22841,7 +22841,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="245">
+    <row r="245" hidden="1">
       <c r="A245" s="3" t="s">
         <v>644</v>
       </c>
@@ -22983,7 +22983,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="247">
+    <row r="247" hidden="1">
       <c r="A247" s="3" t="s">
         <v>644</v>
       </c>
@@ -23055,7 +23055,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="248">
+    <row r="248" hidden="1">
       <c r="A248" s="3" t="s">
         <v>644</v>
       </c>
@@ -23127,7 +23127,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="249">
+    <row r="249" hidden="1">
       <c r="A249" s="3" t="s">
         <v>644</v>
       </c>
@@ -23197,7 +23197,7 @@
       </c>
       <c r="W249" s="7"/>
     </row>
-    <row r="250">
+    <row r="250" hidden="1">
       <c r="A250" s="3" t="s">
         <v>644</v>
       </c>
@@ -23269,7 +23269,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="251">
+    <row r="251" hidden="1">
       <c r="A251" s="3" t="s">
         <v>672</v>
       </c>
@@ -23341,7 +23341,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="252">
+    <row r="252" hidden="1">
       <c r="A252" s="3" t="s">
         <v>672</v>
       </c>
@@ -23413,7 +23413,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" hidden="1">
       <c r="A253" s="3" t="s">
         <v>672</v>
       </c>
@@ -23485,7 +23485,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="254">
+    <row r="254" hidden="1">
       <c r="A254" s="3" t="s">
         <v>679</v>
       </c>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="W254" s="7"/>
     </row>
-    <row r="255">
+    <row r="255" hidden="1">
       <c r="A255" s="3" t="s">
         <v>679</v>
       </c>
@@ -23621,7 +23621,7 @@
       </c>
       <c r="W255" s="7"/>
     </row>
-    <row r="256">
+    <row r="256" hidden="1">
       <c r="A256" s="3" t="s">
         <v>684</v>
       </c>
@@ -23693,7 +23693,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="257">
+    <row r="257" hidden="1">
       <c r="A257" s="3" t="s">
         <v>687</v>
       </c>
@@ -23761,7 +23761,7 @@
       </c>
       <c r="W257" s="7"/>
     </row>
-    <row r="258">
+    <row r="258" hidden="1">
       <c r="A258" s="3" t="s">
         <v>690</v>
       </c>
@@ -23903,7 +23903,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" hidden="1">
       <c r="A260" s="3" t="s">
         <v>694</v>
       </c>
@@ -23975,7 +23975,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="261">
+    <row r="261" hidden="1">
       <c r="A261" s="3" t="s">
         <v>696</v>
       </c>
@@ -24043,7 +24043,7 @@
       </c>
       <c r="W261" s="7"/>
     </row>
-    <row r="262">
+    <row r="262" hidden="1">
       <c r="A262" s="3" t="s">
         <v>699</v>
       </c>
@@ -24115,7 +24115,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" hidden="1">
       <c r="A263" s="3" t="s">
         <v>702</v>
       </c>
@@ -24187,7 +24187,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="264">
+    <row r="264" hidden="1">
       <c r="A264" s="3" t="s">
         <v>705</v>
       </c>
@@ -24259,7 +24259,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="265">
+    <row r="265" hidden="1">
       <c r="A265" s="3" t="s">
         <v>708</v>
       </c>
@@ -24331,7 +24331,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="266">
+    <row r="266" hidden="1">
       <c r="A266" s="3" t="s">
         <v>711</v>
       </c>
@@ -24399,7 +24399,7 @@
       </c>
       <c r="W266" s="7"/>
     </row>
-    <row r="267">
+    <row r="267" hidden="1">
       <c r="A267" s="3" t="s">
         <v>713</v>
       </c>
@@ -24467,7 +24467,7 @@
       </c>
       <c r="W267" s="7"/>
     </row>
-    <row r="268">
+    <row r="268" hidden="1">
       <c r="A268" s="3" t="s">
         <v>716</v>
       </c>
@@ -24539,7 +24539,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="269">
+    <row r="269" hidden="1">
       <c r="A269" s="3" t="s">
         <v>719</v>
       </c>
@@ -24607,7 +24607,7 @@
       </c>
       <c r="W269" s="7"/>
     </row>
-    <row r="270">
+    <row r="270" hidden="1">
       <c r="A270" s="3" t="s">
         <v>722</v>
       </c>
@@ -24675,7 +24675,7 @@
       </c>
       <c r="W270" s="7"/>
     </row>
-    <row r="271">
+    <row r="271" hidden="1">
       <c r="A271" s="3" t="s">
         <v>725</v>
       </c>
@@ -24817,7 +24817,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="273">
+    <row r="273" hidden="1">
       <c r="A273" s="3" t="s">
         <v>731</v>
       </c>
@@ -24889,7 +24889,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="274">
+    <row r="274" hidden="1">
       <c r="A274" s="3" t="s">
         <v>733</v>
       </c>
@@ -25027,7 +25027,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="276">
+    <row r="276" hidden="1">
       <c r="A276" s="3" t="s">
         <v>738</v>
       </c>
@@ -25095,7 +25095,7 @@
       </c>
       <c r="W276" s="7"/>
     </row>
-    <row r="277">
+    <row r="277" hidden="1">
       <c r="A277" s="3" t="s">
         <v>741</v>
       </c>
@@ -25167,7 +25167,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="278">
+    <row r="278" hidden="1">
       <c r="A278" s="3" t="s">
         <v>744</v>
       </c>
@@ -25239,7 +25239,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="279">
+    <row r="279" hidden="1">
       <c r="A279" s="3" t="s">
         <v>747</v>
       </c>
@@ -25307,7 +25307,7 @@
       </c>
       <c r="W279" s="7"/>
     </row>
-    <row r="280">
+    <row r="280" hidden="1">
       <c r="A280" s="3" t="s">
         <v>750</v>
       </c>
@@ -25379,7 +25379,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="281">
+    <row r="281" hidden="1">
       <c r="A281" s="3" t="s">
         <v>753</v>
       </c>
@@ -25451,7 +25451,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="282">
+    <row r="282" hidden="1">
       <c r="A282" s="3" t="s">
         <v>756</v>
       </c>
@@ -25523,7 +25523,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="283">
+    <row r="283" hidden="1">
       <c r="A283" s="3" t="s">
         <v>759</v>
       </c>
@@ -25595,7 +25595,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="284">
+    <row r="284" hidden="1">
       <c r="A284" s="3" t="s">
         <v>762</v>
       </c>
@@ -25667,7 +25667,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="285">
+    <row r="285" hidden="1">
       <c r="A285" s="3" t="s">
         <v>762</v>
       </c>
@@ -25879,7 +25879,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="288">
+    <row r="288" hidden="1">
       <c r="A288" s="3" t="s">
         <v>772</v>
       </c>
@@ -26017,7 +26017,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="290">
+    <row r="290" hidden="1">
       <c r="A290" s="3" t="s">
         <v>778</v>
       </c>
@@ -26089,7 +26089,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="291">
+    <row r="291" hidden="1">
       <c r="A291" s="3" t="s">
         <v>781</v>
       </c>
@@ -26227,7 +26227,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="293">
+    <row r="293" hidden="1">
       <c r="A293" s="3" t="s">
         <v>787</v>
       </c>
@@ -26299,7 +26299,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="294">
+    <row r="294" hidden="1">
       <c r="A294" s="3" t="s">
         <v>790</v>
       </c>
@@ -26367,7 +26367,7 @@
       </c>
       <c r="W294" s="7"/>
     </row>
-    <row r="295">
+    <row r="295" hidden="1">
       <c r="A295" s="3" t="s">
         <v>793</v>
       </c>
@@ -26435,7 +26435,7 @@
       </c>
       <c r="W295" s="7"/>
     </row>
-    <row r="296">
+    <row r="296" hidden="1">
       <c r="A296" s="3" t="s">
         <v>796</v>
       </c>
@@ -26507,7 +26507,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="297">
+    <row r="297" hidden="1">
       <c r="A297" s="3" t="s">
         <v>799</v>
       </c>
@@ -26579,7 +26579,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="298">
+    <row r="298" hidden="1">
       <c r="A298" s="3" t="s">
         <v>802</v>
       </c>
@@ -26651,7 +26651,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="299">
+    <row r="299" hidden="1">
       <c r="A299" s="3" t="s">
         <v>805</v>
       </c>
@@ -26723,7 +26723,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="300">
+    <row r="300" hidden="1">
       <c r="A300" s="3" t="s">
         <v>808</v>
       </c>
@@ -26795,7 +26795,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="301">
+    <row r="301" hidden="1">
       <c r="A301" s="3" t="s">
         <v>810</v>
       </c>
@@ -26863,7 +26863,7 @@
       </c>
       <c r="W301" s="7"/>
     </row>
-    <row r="302">
+    <row r="302" hidden="1">
       <c r="A302" s="3" t="s">
         <v>814</v>
       </c>
@@ -27005,7 +27005,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="304">
+    <row r="304" hidden="1">
       <c r="A304" s="3" t="s">
         <v>820</v>
       </c>
@@ -27077,7 +27077,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="305">
+    <row r="305" hidden="1">
       <c r="A305" s="3" t="s">
         <v>823</v>
       </c>
@@ -27149,7 +27149,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="306">
+    <row r="306" hidden="1">
       <c r="A306" s="3" t="s">
         <v>826</v>
       </c>
@@ -27217,7 +27217,7 @@
       </c>
       <c r="W306" s="7"/>
     </row>
-    <row r="307">
+    <row r="307" hidden="1">
       <c r="A307" s="3" t="s">
         <v>829</v>
       </c>
@@ -27289,7 +27289,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="308">
+    <row r="308" hidden="1">
       <c r="A308" s="3" t="s">
         <v>831</v>
       </c>
@@ -27361,7 +27361,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="309">
+    <row r="309" hidden="1">
       <c r="A309" s="3" t="s">
         <v>833</v>
       </c>
@@ -27433,7 +27433,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="310">
+    <row r="310" hidden="1">
       <c r="A310" s="3" t="s">
         <v>836</v>
       </c>
@@ -27505,7 +27505,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="311">
+    <row r="311" hidden="1">
       <c r="A311" s="3" t="s">
         <v>839</v>
       </c>
@@ -27647,7 +27647,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="313">
+    <row r="313" hidden="1">
       <c r="A313" s="3" t="s">
         <v>841</v>
       </c>
@@ -27719,7 +27719,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="314">
+    <row r="314" hidden="1">
       <c r="A314" s="3" t="s">
         <v>841</v>
       </c>
@@ -27791,7 +27791,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="315">
+    <row r="315" hidden="1">
       <c r="A315" s="3" t="s">
         <v>841</v>
       </c>
@@ -27933,7 +27933,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="317">
+    <row r="317" hidden="1">
       <c r="A317" s="3" t="s">
         <v>853</v>
       </c>
@@ -28005,7 +28005,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="318">
+    <row r="318" hidden="1">
       <c r="A318" s="3" t="s">
         <v>856</v>
       </c>
@@ -28077,7 +28077,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="319">
+    <row r="319" hidden="1">
       <c r="A319" s="3" t="s">
         <v>859</v>
       </c>
@@ -28145,7 +28145,7 @@
       </c>
       <c r="W319" s="7"/>
     </row>
-    <row r="320">
+    <row r="320" hidden="1">
       <c r="A320" s="3" t="s">
         <v>859</v>
       </c>
@@ -28217,7 +28217,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="321">
+    <row r="321" hidden="1">
       <c r="A321" s="3" t="s">
         <v>859</v>
       </c>
@@ -28285,7 +28285,7 @@
       </c>
       <c r="W321" s="7"/>
     </row>
-    <row r="322">
+    <row r="322" hidden="1">
       <c r="A322" s="3" t="s">
         <v>859</v>
       </c>
@@ -28357,7 +28357,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="323">
+    <row r="323" hidden="1">
       <c r="A323" s="3" t="s">
         <v>868</v>
       </c>
@@ -28429,7 +28429,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="324">
+    <row r="324" hidden="1">
       <c r="A324" s="3" t="s">
         <v>871</v>
       </c>
@@ -28501,7 +28501,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="325">
+    <row r="325" hidden="1">
       <c r="A325" s="3" t="s">
         <v>874</v>
       </c>
@@ -28573,7 +28573,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="326">
+    <row r="326" hidden="1">
       <c r="A326" s="3" t="s">
         <v>877</v>
       </c>
@@ -28641,7 +28641,7 @@
       </c>
       <c r="W326" s="7"/>
     </row>
-    <row r="327">
+    <row r="327" hidden="1">
       <c r="A327" s="3" t="s">
         <v>877</v>
       </c>
@@ -28713,7 +28713,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="328">
+    <row r="328" hidden="1">
       <c r="A328" s="3" t="s">
         <v>881</v>
       </c>
@@ -28785,7 +28785,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="329">
+    <row r="329" hidden="1">
       <c r="A329" s="3" t="s">
         <v>884</v>
       </c>
@@ -28857,7 +28857,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="330">
+    <row r="330" hidden="1">
       <c r="A330" s="3" t="s">
         <v>887</v>
       </c>
@@ -28999,7 +28999,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="332">
+    <row r="332" hidden="1">
       <c r="A332" s="3" t="s">
         <v>891</v>
       </c>
@@ -29071,7 +29071,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="333">
+    <row r="333" hidden="1">
       <c r="A333" s="3" t="s">
         <v>892</v>
       </c>
@@ -29213,7 +29213,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="335">
+    <row r="335" hidden="1">
       <c r="A335" s="3" t="s">
         <v>898</v>
       </c>
@@ -29285,7 +29285,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="336">
+    <row r="336" hidden="1">
       <c r="A336" s="3" t="s">
         <v>901</v>
       </c>
@@ -29357,7 +29357,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="337">
+    <row r="337" hidden="1">
       <c r="A337" s="3" t="s">
         <v>904</v>
       </c>
@@ -29425,7 +29425,7 @@
       </c>
       <c r="W337" s="7"/>
     </row>
-    <row r="338">
+    <row r="338" hidden="1">
       <c r="A338" s="3" t="s">
         <v>907</v>
       </c>
@@ -29637,7 +29637,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="341">
+    <row r="341" hidden="1">
       <c r="A341" s="3" t="s">
         <v>916</v>
       </c>
@@ -29709,7 +29709,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="342">
+    <row r="342" hidden="1">
       <c r="A342" s="3" t="s">
         <v>916</v>
       </c>
@@ -29781,7 +29781,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="343">
+    <row r="343" hidden="1">
       <c r="A343" s="3" t="s">
         <v>921</v>
       </c>
@@ -29849,7 +29849,7 @@
       </c>
       <c r="W343" s="7"/>
     </row>
-    <row r="344">
+    <row r="344" hidden="1">
       <c r="A344" s="3" t="s">
         <v>924</v>
       </c>
@@ -29917,7 +29917,7 @@
       </c>
       <c r="W344" s="7"/>
     </row>
-    <row r="345">
+    <row r="345" hidden="1">
       <c r="A345" s="3" t="s">
         <v>927</v>
       </c>
@@ -29985,7 +29985,7 @@
       </c>
       <c r="W345" s="7"/>
     </row>
-    <row r="346">
+    <row r="346" hidden="1">
       <c r="A346" s="3" t="s">
         <v>930</v>
       </c>
@@ -30053,7 +30053,7 @@
       </c>
       <c r="W346" s="7"/>
     </row>
-    <row r="347">
+    <row r="347" hidden="1">
       <c r="A347" s="3" t="s">
         <v>933</v>
       </c>
@@ -30121,7 +30121,7 @@
       </c>
       <c r="W347" s="7"/>
     </row>
-    <row r="348">
+    <row r="348" hidden="1">
       <c r="A348" s="3" t="s">
         <v>936</v>
       </c>
@@ -30193,7 +30193,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="349">
+    <row r="349" hidden="1">
       <c r="A349" s="3" t="s">
         <v>938</v>
       </c>
@@ -30265,7 +30265,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="350">
+    <row r="350" hidden="1">
       <c r="A350" s="3" t="s">
         <v>941</v>
       </c>
@@ -30337,7 +30337,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="351">
+    <row r="351" hidden="1">
       <c r="A351" s="3" t="s">
         <v>944</v>
       </c>
@@ -30409,7 +30409,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="352">
+    <row r="352" hidden="1">
       <c r="A352" s="3" t="s">
         <v>946</v>
       </c>
@@ -30547,7 +30547,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="354">
+    <row r="354" hidden="1">
       <c r="A354" s="3" t="s">
         <v>949</v>
       </c>
@@ -30619,7 +30619,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="355">
+    <row r="355" hidden="1">
       <c r="A355" s="3" t="s">
         <v>949</v>
       </c>
@@ -30761,7 +30761,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="357">
+    <row r="357" hidden="1">
       <c r="A357" s="3" t="s">
         <v>958</v>
       </c>
@@ -30833,7 +30833,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="358">
+    <row r="358" hidden="1">
       <c r="A358" s="3" t="s">
         <v>958</v>
       </c>
@@ -30905,7 +30905,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="359">
+    <row r="359" hidden="1">
       <c r="A359" s="3" t="s">
         <v>963</v>
       </c>
@@ -30977,7 +30977,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="360">
+    <row r="360" hidden="1">
       <c r="A360" s="3" t="s">
         <v>966</v>
       </c>
@@ -31049,7 +31049,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="361">
+    <row r="361" hidden="1">
       <c r="A361" s="3" t="s">
         <v>969</v>
       </c>
@@ -31121,7 +31121,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="362">
+    <row r="362" hidden="1">
       <c r="A362" s="3" t="s">
         <v>972</v>
       </c>
@@ -31193,7 +31193,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="363">
+    <row r="363" hidden="1">
       <c r="A363" s="3" t="s">
         <v>975</v>
       </c>
@@ -31261,7 +31261,7 @@
       </c>
       <c r="W363" s="7"/>
     </row>
-    <row r="364">
+    <row r="364" hidden="1">
       <c r="A364" s="3" t="s">
         <v>549</v>
       </c>
@@ -31333,7 +31333,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="365">
+    <row r="365" hidden="1">
       <c r="A365" s="3" t="s">
         <v>980</v>
       </c>
@@ -31405,7 +31405,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="366">
+    <row r="366" hidden="1">
       <c r="A366" s="3" t="s">
         <v>983</v>
       </c>
@@ -31477,7 +31477,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="367">
+    <row r="367" hidden="1">
       <c r="A367" s="3" t="s">
         <v>986</v>
       </c>
@@ -31549,7 +31549,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="368">
+    <row r="368" hidden="1">
       <c r="A368" s="3" t="s">
         <v>989</v>
       </c>
@@ -31621,7 +31621,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="369">
+    <row r="369" hidden="1">
       <c r="A369" s="3" t="s">
         <v>992</v>
       </c>
@@ -31693,7 +31693,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="370">
+    <row r="370" hidden="1">
       <c r="A370" s="3" t="s">
         <v>995</v>
       </c>
@@ -31765,7 +31765,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="371">
+    <row r="371" hidden="1">
       <c r="A371" s="3" t="s">
         <v>997</v>
       </c>
@@ -31837,7 +31837,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="372">
+    <row r="372" hidden="1">
       <c r="A372" s="3" t="s">
         <v>1000</v>
       </c>
@@ -31907,7 +31907,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="373">
+    <row r="373" hidden="1">
       <c r="A373" s="3" t="s">
         <v>1002</v>
       </c>
@@ -31979,7 +31979,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="374">
+    <row r="374" hidden="1">
       <c r="A374" s="3" t="s">
         <v>1005</v>
       </c>
@@ -32051,7 +32051,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="375">
+    <row r="375" hidden="1">
       <c r="A375" s="3" t="s">
         <v>1005</v>
       </c>
@@ -32123,7 +32123,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="376">
+    <row r="376" hidden="1">
       <c r="A376" s="3" t="s">
         <v>1010</v>
       </c>
@@ -32261,7 +32261,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="378">
+    <row r="378" hidden="1">
       <c r="A378" s="3" t="s">
         <v>1015</v>
       </c>
@@ -32329,7 +32329,7 @@
       </c>
       <c r="W378" s="7"/>
     </row>
-    <row r="379">
+    <row r="379" hidden="1">
       <c r="A379" s="3" t="s">
         <v>1018</v>
       </c>
@@ -32401,7 +32401,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="380">
+    <row r="380" hidden="1">
       <c r="A380" s="3" t="s">
         <v>1021</v>
       </c>
@@ -32473,7 +32473,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="381">
+    <row r="381" hidden="1">
       <c r="A381" s="3" t="s">
         <v>1024</v>
       </c>
@@ -32545,7 +32545,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="382">
+    <row r="382" hidden="1">
       <c r="A382" s="3" t="s">
         <v>1027</v>
       </c>
@@ -32617,7 +32617,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="383">
+    <row r="383" hidden="1">
       <c r="A383" s="3" t="s">
         <v>1030</v>
       </c>
@@ -32829,7 +32829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="386">
+    <row r="386" hidden="1">
       <c r="A386" s="3" t="s">
         <v>1039</v>
       </c>
@@ -32901,7 +32901,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="387">
+    <row r="387" hidden="1">
       <c r="A387" s="3" t="s">
         <v>1041</v>
       </c>
@@ -32973,7 +32973,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="388">
+    <row r="388" hidden="1">
       <c r="A388" s="3" t="s">
         <v>1043</v>
       </c>
@@ -33045,7 +33045,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="389">
+    <row r="389" hidden="1">
       <c r="A389" s="3" t="s">
         <v>1046</v>
       </c>
@@ -33117,7 +33117,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="390">
+    <row r="390" hidden="1">
       <c r="A390" s="3" t="s">
         <v>1049</v>
       </c>
@@ -33185,7 +33185,7 @@
       </c>
       <c r="W390" s="7"/>
     </row>
-    <row r="391">
+    <row r="391" hidden="1">
       <c r="A391" s="3" t="s">
         <v>1051</v>
       </c>
@@ -33257,7 +33257,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="392">
+    <row r="392" hidden="1">
       <c r="A392" s="3" t="s">
         <v>1054</v>
       </c>
@@ -33329,7 +33329,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="393">
+    <row r="393" hidden="1">
       <c r="A393" s="3" t="s">
         <v>1057</v>
       </c>
@@ -33401,7 +33401,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="394">
+    <row r="394" hidden="1">
       <c r="A394" s="3" t="s">
         <v>1060</v>
       </c>
@@ -33543,7 +33543,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="396">
+    <row r="396" hidden="1">
       <c r="A396" s="3" t="s">
         <v>1065</v>
       </c>
@@ -33615,7 +33615,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="397">
+    <row r="397" hidden="1">
       <c r="A397" s="3" t="s">
         <v>1066</v>
       </c>
@@ -33687,7 +33687,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="398">
+    <row r="398" hidden="1">
       <c r="A398" s="3" t="s">
         <v>1068</v>
       </c>
@@ -33755,7 +33755,7 @@
       </c>
       <c r="W398" s="7"/>
     </row>
-    <row r="399">
+    <row r="399" hidden="1">
       <c r="A399" s="3" t="s">
         <v>1071</v>
       </c>
@@ -33823,7 +33823,7 @@
       </c>
       <c r="W399" s="7"/>
     </row>
-    <row r="400">
+    <row r="400" hidden="1">
       <c r="A400" s="3" t="s">
         <v>1071</v>
       </c>
@@ -34035,7 +34035,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="403">
+    <row r="403" hidden="1">
       <c r="A403" s="3" t="s">
         <v>1082</v>
       </c>
@@ -34107,7 +34107,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="404">
+    <row r="404" hidden="1">
       <c r="A404" s="3" t="s">
         <v>1085</v>
       </c>
@@ -34175,7 +34175,7 @@
       </c>
       <c r="W404" s="7"/>
     </row>
-    <row r="405">
+    <row r="405" hidden="1">
       <c r="A405" s="3" t="s">
         <v>1088</v>
       </c>
@@ -34247,7 +34247,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="406">
+    <row r="406" hidden="1">
       <c r="A406" s="3" t="s">
         <v>1091</v>
       </c>
@@ -34319,7 +34319,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="407">
+    <row r="407" hidden="1">
       <c r="A407" s="3" t="s">
         <v>1094</v>
       </c>
@@ -34387,7 +34387,7 @@
       </c>
       <c r="W407" s="7"/>
     </row>
-    <row r="408">
+    <row r="408" hidden="1">
       <c r="A408" s="3" t="s">
         <v>1094</v>
       </c>
@@ -34455,7 +34455,7 @@
       </c>
       <c r="W408" s="7"/>
     </row>
-    <row r="409">
+    <row r="409" hidden="1">
       <c r="A409" s="3" t="s">
         <v>1099</v>
       </c>
@@ -34525,7 +34525,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="410">
+    <row r="410" hidden="1">
       <c r="A410" s="3" t="s">
         <v>1101</v>
       </c>
@@ -34597,7 +34597,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="411">
+    <row r="411" hidden="1">
       <c r="A411" s="3" t="s">
         <v>1104</v>
       </c>
@@ -34669,7 +34669,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="412">
+    <row r="412" hidden="1">
       <c r="A412" s="3" t="s">
         <v>1104</v>
       </c>
@@ -34741,7 +34741,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="413">
+    <row r="413" hidden="1">
       <c r="A413" s="3" t="s">
         <v>1109</v>
       </c>
@@ -34813,7 +34813,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="414">
+    <row r="414" hidden="1">
       <c r="A414" s="3" t="s">
         <v>1112</v>
       </c>
@@ -34881,7 +34881,7 @@
       </c>
       <c r="W414" s="7"/>
     </row>
-    <row r="415">
+    <row r="415" hidden="1">
       <c r="A415" s="3" t="s">
         <v>1114</v>
       </c>
@@ -34953,7 +34953,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="416">
+    <row r="416" hidden="1">
       <c r="A416" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35025,7 +35025,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="417">
+    <row r="417" hidden="1">
       <c r="A417" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35097,7 +35097,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="418">
+    <row r="418" hidden="1">
       <c r="A418" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35169,7 +35169,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="419">
+    <row r="419" hidden="1">
       <c r="A419" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35237,7 +35237,7 @@
       </c>
       <c r="W419" s="7"/>
     </row>
-    <row r="420">
+    <row r="420" hidden="1">
       <c r="A420" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35309,7 +35309,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="421">
+    <row r="421" hidden="1">
       <c r="A421" s="3" t="s">
         <v>1117</v>
       </c>
@@ -35381,7 +35381,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="422">
+    <row r="422" hidden="1">
       <c r="A422" s="3" t="s">
         <v>1130</v>
       </c>
@@ -35523,7 +35523,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="424">
+    <row r="424" hidden="1">
       <c r="A424" s="3" t="s">
         <v>1135</v>
       </c>
@@ -35595,7 +35595,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="425">
+    <row r="425" hidden="1">
       <c r="A425" s="3" t="s">
         <v>1137</v>
       </c>
@@ -35667,7 +35667,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="426">
+    <row r="426" hidden="1">
       <c r="A426" s="3" t="s">
         <v>1140</v>
       </c>
@@ -35739,7 +35739,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="427">
+    <row r="427" hidden="1">
       <c r="A427" s="3" t="s">
         <v>1143</v>
       </c>
@@ -35881,7 +35881,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="429">
+    <row r="429" hidden="1">
       <c r="A429" s="3" t="s">
         <v>1149</v>
       </c>
@@ -35949,7 +35949,7 @@
       </c>
       <c r="W429" s="7"/>
     </row>
-    <row r="430">
+    <row r="430" hidden="1">
       <c r="A430" s="3" t="s">
         <v>1151</v>
       </c>
@@ -36021,7 +36021,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="431">
+    <row r="431" hidden="1">
       <c r="A431" s="3" t="s">
         <v>1154</v>
       </c>
@@ -36093,7 +36093,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="432">
+    <row r="432" hidden="1">
       <c r="A432" s="3" t="s">
         <v>1156</v>
       </c>
@@ -36165,7 +36165,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="433">
+    <row r="433" hidden="1">
       <c r="A433" s="26" t="s">
         <v>1159</v>
       </c>
@@ -36233,7 +36233,7 @@
       </c>
       <c r="W433" s="7"/>
     </row>
-    <row r="434">
+    <row r="434" hidden="1">
       <c r="A434" s="26" t="s">
         <v>1159</v>
       </c>
@@ -36301,7 +36301,7 @@
       </c>
       <c r="W434" s="7"/>
     </row>
-    <row r="435">
+    <row r="435" hidden="1">
       <c r="A435" s="3" t="s">
         <v>1164</v>
       </c>
@@ -36443,7 +36443,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="437">
+    <row r="437" hidden="1">
       <c r="A437" s="3" t="s">
         <v>1169</v>
       </c>
@@ -36655,7 +36655,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="440">
+    <row r="440" hidden="1">
       <c r="A440" s="3" t="s">
         <v>1177</v>
       </c>
@@ -36727,7 +36727,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="441">
+    <row r="441" hidden="1">
       <c r="A441" s="3" t="s">
         <v>1180</v>
       </c>
@@ -36799,7 +36799,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="442">
+    <row r="442" hidden="1">
       <c r="A442" s="3" t="s">
         <v>1183</v>
       </c>
@@ -36941,7 +36941,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="444">
+    <row r="444" hidden="1">
       <c r="A444" s="3" t="s">
         <v>1188</v>
       </c>
@@ -37013,7 +37013,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="445">
+    <row r="445" hidden="1">
       <c r="A445" s="3" t="s">
         <v>1188</v>
       </c>
@@ -37085,7 +37085,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="446">
+    <row r="446" hidden="1">
       <c r="A446" s="3" t="s">
         <v>1188</v>
       </c>
@@ -37157,7 +37157,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="447">
+    <row r="447" hidden="1">
       <c r="A447" s="3" t="s">
         <v>1195</v>
       </c>
@@ -37225,7 +37225,7 @@
       </c>
       <c r="W447" s="7"/>
     </row>
-    <row r="448">
+    <row r="448" hidden="1">
       <c r="A448" s="3" t="s">
         <v>1198</v>
       </c>
@@ -37293,7 +37293,7 @@
       </c>
       <c r="W448" s="7"/>
     </row>
-    <row r="449">
+    <row r="449" hidden="1">
       <c r="A449" s="3" t="s">
         <v>1201</v>
       </c>
@@ -37361,7 +37361,7 @@
       </c>
       <c r="W449" s="7"/>
     </row>
-    <row r="450">
+    <row r="450" hidden="1">
       <c r="A450" s="3" t="s">
         <v>1204</v>
       </c>
@@ -37433,7 +37433,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="451">
+    <row r="451" hidden="1">
       <c r="A451" s="3" t="s">
         <v>1206</v>
       </c>
@@ -37501,7 +37501,7 @@
       </c>
       <c r="W451" s="7"/>
     </row>
-    <row r="452">
+    <row r="452" hidden="1">
       <c r="A452" s="3" t="s">
         <v>1206</v>
       </c>
@@ -37573,7 +37573,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="453">
+    <row r="453" hidden="1">
       <c r="A453" s="3" t="s">
         <v>1209</v>
       </c>
@@ -37645,7 +37645,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="454">
+    <row r="454" hidden="1">
       <c r="A454" s="3" t="s">
         <v>1211</v>
       </c>
@@ -37713,7 +37713,7 @@
       </c>
       <c r="W454" s="7"/>
     </row>
-    <row r="455">
+    <row r="455" hidden="1">
       <c r="A455" s="3" t="s">
         <v>1213</v>
       </c>
@@ -37785,7 +37785,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="456">
+    <row r="456" hidden="1">
       <c r="A456" s="3" t="s">
         <v>1215</v>
       </c>
@@ -37857,7 +37857,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="457">
+    <row r="457" hidden="1">
       <c r="A457" s="3" t="s">
         <v>1217</v>
       </c>
@@ -37929,7 +37929,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="458">
+    <row r="458" hidden="1">
       <c r="A458" s="3" t="s">
         <v>1220</v>
       </c>
@@ -38001,7 +38001,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="459">
+    <row r="459" hidden="1">
       <c r="A459" s="3" t="s">
         <v>1223</v>
       </c>
@@ -38073,7 +38073,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="460">
+    <row r="460" hidden="1">
       <c r="A460" s="3" t="s">
         <v>1226</v>
       </c>
@@ -38141,7 +38141,7 @@
       </c>
       <c r="W460" s="7"/>
     </row>
-    <row r="461">
+    <row r="461" hidden="1">
       <c r="A461" s="3" t="s">
         <v>1229</v>
       </c>
@@ -38213,7 +38213,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="462">
+    <row r="462" hidden="1">
       <c r="A462" s="3" t="s">
         <v>1232</v>
       </c>
@@ -38285,7 +38285,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="463">
+    <row r="463" hidden="1">
       <c r="A463" s="3" t="s">
         <v>1235</v>
       </c>
@@ -38357,7 +38357,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="464">
+    <row r="464" hidden="1">
       <c r="A464" s="3" t="s">
         <v>1237</v>
       </c>
@@ -38429,7 +38429,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="465">
+    <row r="465" hidden="1">
       <c r="A465" s="3" t="s">
         <v>1240</v>
       </c>
@@ -38501,7 +38501,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="466">
+    <row r="466" hidden="1">
       <c r="A466" s="3" t="s">
         <v>1242</v>
       </c>
@@ -38713,7 +38713,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="469">
+    <row r="469" hidden="1">
       <c r="A469" s="3" t="s">
         <v>1249</v>
       </c>
@@ -38785,7 +38785,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="470">
+    <row r="470" hidden="1">
       <c r="A470" s="3" t="s">
         <v>1251</v>
       </c>
@@ -38927,7 +38927,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="472">
+    <row r="472" hidden="1">
       <c r="A472" s="3" t="s">
         <v>1255</v>
       </c>
@@ -38999,7 +38999,7 @@
         <v>1258</v>
       </c>
     </row>
-    <row r="473">
+    <row r="473" hidden="1">
       <c r="A473" s="3" t="s">
         <v>1259</v>
       </c>
@@ -39071,7 +39071,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="474">
+    <row r="474" hidden="1">
       <c r="A474" s="3" t="s">
         <v>1262</v>
       </c>
@@ -39143,7 +39143,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="475">
+    <row r="475" hidden="1">
       <c r="A475" s="3" t="s">
         <v>1265</v>
       </c>
@@ -39285,7 +39285,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="477">
+    <row r="477" hidden="1">
       <c r="A477" s="3" t="s">
         <v>1270</v>
       </c>
@@ -39357,7 +39357,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="478">
+    <row r="478" hidden="1">
       <c r="A478" s="3" t="s">
         <v>1273</v>
       </c>
@@ -39429,7 +39429,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="479">
+    <row r="479" hidden="1">
       <c r="A479" s="3" t="s">
         <v>1273</v>
       </c>
@@ -39501,7 +39501,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="480">
+    <row r="480" hidden="1">
       <c r="A480" s="3" t="s">
         <v>1278</v>
       </c>
@@ -39573,7 +39573,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="481">
+    <row r="481" hidden="1">
       <c r="A481" s="3" t="s">
         <v>1280</v>
       </c>
@@ -39645,7 +39645,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="482">
+    <row r="482" hidden="1">
       <c r="A482" s="3" t="s">
         <v>1282</v>
       </c>
@@ -39713,7 +39713,7 @@
       </c>
       <c r="W482" s="7"/>
     </row>
-    <row r="483">
+    <row r="483" hidden="1">
       <c r="A483" s="3" t="s">
         <v>1285</v>
       </c>
@@ -39855,7 +39855,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="485">
+    <row r="485" hidden="1">
       <c r="A485" s="3" t="s">
         <v>1290</v>
       </c>
@@ -39927,7 +39927,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="486">
+    <row r="486" hidden="1">
       <c r="A486" s="30" t="s">
         <v>1292</v>
       </c>
@@ -39995,7 +39995,7 @@
       </c>
       <c r="W486" s="7"/>
     </row>
-    <row r="487">
+    <row r="487" hidden="1">
       <c r="A487" s="3" t="s">
         <v>1292</v>
       </c>
@@ -40063,7 +40063,7 @@
       </c>
       <c r="W487" s="7"/>
     </row>
-    <row r="488">
+    <row r="488" hidden="1">
       <c r="A488" s="3" t="s">
         <v>1292</v>
       </c>
@@ -40135,7 +40135,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="489">
+    <row r="489" hidden="1">
       <c r="A489" s="3" t="s">
         <v>1297</v>
       </c>
@@ -40207,7 +40207,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="490">
+    <row r="490" hidden="1">
       <c r="A490" s="3" t="s">
         <v>1293</v>
       </c>
@@ -40275,7 +40275,7 @@
       </c>
       <c r="W490" s="7"/>
     </row>
-    <row r="491">
+    <row r="491" hidden="1">
       <c r="A491" s="3" t="s">
         <v>1299</v>
       </c>
@@ -40347,7 +40347,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="492">
+    <row r="492" hidden="1">
       <c r="A492" s="3" t="s">
         <v>1302</v>
       </c>
@@ -40419,7 +40419,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="493">
+    <row r="493" hidden="1">
       <c r="A493" s="3" t="s">
         <v>1302</v>
       </c>
@@ -40491,7 +40491,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="494">
+    <row r="494" hidden="1">
       <c r="A494" s="3" t="s">
         <v>1307</v>
       </c>
@@ -40563,7 +40563,7 @@
         <v>1258</v>
       </c>
     </row>
-    <row r="495">
+    <row r="495" hidden="1">
       <c r="A495" s="3" t="s">
         <v>1307</v>
       </c>
@@ -40635,7 +40635,7 @@
         <v>1258</v>
       </c>
     </row>
-    <row r="496">
+    <row r="496" hidden="1">
       <c r="A496" s="3" t="s">
         <v>1307</v>
       </c>
@@ -40707,7 +40707,7 @@
         <v>1258</v>
       </c>
     </row>
-    <row r="497">
+    <row r="497" hidden="1">
       <c r="A497" s="3" t="s">
         <v>1314</v>
       </c>
@@ -40845,7 +40845,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="499">
+    <row r="499" hidden="1">
       <c r="A499" s="3" t="s">
         <v>1319</v>
       </c>
@@ -40917,7 +40917,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="500">
+    <row r="500" hidden="1">
       <c r="A500" s="3" t="s">
         <v>1322</v>
       </c>
@@ -40989,7 +40989,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="501">
+    <row r="501" hidden="1">
       <c r="A501" s="3" t="s">
         <v>1323</v>
       </c>
@@ -41061,7 +41061,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="502">
+    <row r="502" hidden="1">
       <c r="A502" s="3" t="s">
         <v>1326</v>
       </c>
@@ -41133,7 +41133,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="503">
+    <row r="503" hidden="1">
       <c r="A503" s="3" t="s">
         <v>1328</v>
       </c>
@@ -41205,7 +41205,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="504">
+    <row r="504" hidden="1">
       <c r="A504" s="3" t="s">
         <v>1331</v>
       </c>
@@ -41277,7 +41277,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="505">
+    <row r="505" hidden="1">
       <c r="A505" s="3" t="s">
         <v>1333</v>
       </c>
@@ -41349,7 +41349,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="506">
+    <row r="506" hidden="1">
       <c r="A506" s="3" t="s">
         <v>1335</v>
       </c>
@@ -41415,7 +41415,7 @@
       </c>
       <c r="W506" s="7"/>
     </row>
-    <row r="507">
+    <row r="507" hidden="1">
       <c r="A507" s="3" t="s">
         <v>1337</v>
       </c>
@@ -41557,7 +41557,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="509">
+    <row r="509" hidden="1">
       <c r="A509" s="3" t="s">
         <v>1341</v>
       </c>
@@ -41629,7 +41629,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="510">
+    <row r="510" hidden="1">
       <c r="A510" s="3" t="s">
         <v>1344</v>
       </c>
@@ -41701,7 +41701,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="511">
+    <row r="511" hidden="1">
       <c r="A511" s="3" t="s">
         <v>1347</v>
       </c>
@@ -41773,7 +41773,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="512">
+    <row r="512" hidden="1">
       <c r="A512" s="3" t="s">
         <v>1350</v>
       </c>
@@ -41841,7 +41841,7 @@
       </c>
       <c r="W512" s="7"/>
     </row>
-    <row r="513">
+    <row r="513" hidden="1">
       <c r="A513" s="3" t="s">
         <v>1353</v>
       </c>
@@ -41913,7 +41913,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="514">
+    <row r="514" hidden="1">
       <c r="A514" s="3" t="s">
         <v>1356</v>
       </c>
@@ -41985,7 +41985,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="515">
+    <row r="515" hidden="1">
       <c r="A515" s="3" t="s">
         <v>1358</v>
       </c>
@@ -42053,7 +42053,7 @@
       </c>
       <c r="W515" s="7"/>
     </row>
-    <row r="516">
+    <row r="516" hidden="1">
       <c r="A516" s="3" t="s">
         <v>1361</v>
       </c>
@@ -42125,7 +42125,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="517">
+    <row r="517" hidden="1">
       <c r="A517" s="3" t="s">
         <v>1363</v>
       </c>
@@ -42197,7 +42197,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="518">
+    <row r="518" hidden="1">
       <c r="A518" s="3" t="s">
         <v>1366</v>
       </c>
@@ -42265,7 +42265,7 @@
       </c>
       <c r="W518" s="7"/>
     </row>
-    <row r="519">
+    <row r="519" hidden="1">
       <c r="A519" s="3" t="s">
         <v>1368</v>
       </c>
@@ -42337,7 +42337,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="520">
+    <row r="520" hidden="1">
       <c r="A520" s="3" t="s">
         <v>1371</v>
       </c>
@@ -42409,7 +42409,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="521">
+    <row r="521" hidden="1">
       <c r="A521" s="3" t="s">
         <v>1374</v>
       </c>
@@ -42477,7 +42477,7 @@
       </c>
       <c r="W521" s="7"/>
     </row>
-    <row r="522">
+    <row r="522" hidden="1">
       <c r="A522" s="3" t="s">
         <v>1377</v>
       </c>
@@ -42549,7 +42549,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="523">
+    <row r="523" hidden="1">
       <c r="A523" s="3" t="s">
         <v>1380</v>
       </c>
@@ -42621,7 +42621,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="524">
+    <row r="524" hidden="1">
       <c r="A524" s="3" t="s">
         <v>1383</v>
       </c>
@@ -42693,7 +42693,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="525">
+    <row r="525" hidden="1">
       <c r="A525" s="3" t="s">
         <v>1386</v>
       </c>
@@ -42765,7 +42765,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="526">
+    <row r="526" hidden="1">
       <c r="A526" s="3" t="s">
         <v>1389</v>
       </c>
@@ -42833,7 +42833,7 @@
       </c>
       <c r="W526" s="7"/>
     </row>
-    <row r="527">
+    <row r="527" hidden="1">
       <c r="A527" s="3" t="s">
         <v>1392</v>
       </c>
@@ -42905,7 +42905,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="528">
+    <row r="528" hidden="1">
       <c r="A528" s="3" t="s">
         <v>1395</v>
       </c>
@@ -42977,7 +42977,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="529">
+    <row r="529" hidden="1">
       <c r="A529" s="3" t="s">
         <v>1396</v>
       </c>
@@ -43045,7 +43045,7 @@
       </c>
       <c r="W529" s="7"/>
     </row>
-    <row r="530">
+    <row r="530" hidden="1">
       <c r="A530" s="3" t="s">
         <v>1399</v>
       </c>
@@ -43187,7 +43187,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="532">
+    <row r="532" hidden="1">
       <c r="A532" s="3" t="s">
         <v>1404</v>
       </c>
@@ -43259,7 +43259,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="533">
+    <row r="533" hidden="1">
       <c r="A533" s="3" t="s">
         <v>1407</v>
       </c>
@@ -43331,7 +43331,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="534">
+    <row r="534" hidden="1">
       <c r="A534" s="3" t="s">
         <v>1407</v>
       </c>
@@ -43399,7 +43399,7 @@
       </c>
       <c r="W534" s="7"/>
     </row>
-    <row r="535">
+    <row r="535" hidden="1">
       <c r="A535" s="3" t="s">
         <v>1412</v>
       </c>
@@ -43471,7 +43471,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="536">
+    <row r="536" hidden="1">
       <c r="A536" s="3" t="s">
         <v>1414</v>
       </c>
@@ -43539,7 +43539,7 @@
       </c>
       <c r="W536" s="7"/>
     </row>
-    <row r="537">
+    <row r="537" hidden="1">
       <c r="A537" s="3" t="s">
         <v>1414</v>
       </c>
@@ -43607,7 +43607,7 @@
       </c>
       <c r="W537" s="7"/>
     </row>
-    <row r="538">
+    <row r="538" hidden="1">
       <c r="A538" s="3" t="s">
         <v>1419</v>
       </c>
@@ -43679,7 +43679,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="539">
+    <row r="539" hidden="1">
       <c r="A539" s="3" t="s">
         <v>1419</v>
       </c>
@@ -43751,7 +43751,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="540">
+    <row r="540" hidden="1">
       <c r="A540" s="3" t="s">
         <v>1419</v>
       </c>
@@ -43823,7 +43823,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="541">
+    <row r="541" hidden="1">
       <c r="A541" s="3" t="s">
         <v>1419</v>
       </c>
@@ -43895,7 +43895,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="542">
+    <row r="542" hidden="1">
       <c r="A542" s="3" t="s">
         <v>1428</v>
       </c>
@@ -43965,7 +43965,7 @@
       </c>
       <c r="W542" s="7"/>
     </row>
-    <row r="543">
+    <row r="543" hidden="1">
       <c r="A543" s="3" t="s">
         <v>1428</v>
       </c>
@@ -44037,7 +44037,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="544">
+    <row r="544" hidden="1">
       <c r="A544" s="3" t="s">
         <v>1428</v>
       </c>
@@ -44105,7 +44105,7 @@
       </c>
       <c r="W544" s="7"/>
     </row>
-    <row r="545">
+    <row r="545" hidden="1">
       <c r="A545" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44175,7 +44175,7 @@
       </c>
       <c r="W545" s="7"/>
     </row>
-    <row r="546">
+    <row r="546" hidden="1">
       <c r="A546" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44243,7 +44243,7 @@
       </c>
       <c r="W546" s="7"/>
     </row>
-    <row r="547">
+    <row r="547" hidden="1">
       <c r="A547" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44311,7 +44311,7 @@
       </c>
       <c r="W547" s="7"/>
     </row>
-    <row r="548">
+    <row r="548" hidden="1">
       <c r="A548" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44453,7 +44453,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="550">
+    <row r="550" hidden="1">
       <c r="A550" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44591,7 +44591,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="552">
+    <row r="552" hidden="1">
       <c r="A552" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44663,7 +44663,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="553">
+    <row r="553" hidden="1">
       <c r="A553" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44735,7 +44735,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="554">
+    <row r="554" hidden="1">
       <c r="A554" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44803,7 +44803,7 @@
       </c>
       <c r="W554" s="7"/>
     </row>
-    <row r="555">
+    <row r="555" hidden="1">
       <c r="A555" s="3" t="s">
         <v>1435</v>
       </c>
@@ -44875,7 +44875,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="556">
+    <row r="556" hidden="1">
       <c r="A556" s="3" t="s">
         <v>1458</v>
       </c>
@@ -45013,7 +45013,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="558">
+    <row r="558" hidden="1">
       <c r="A558" s="3" t="s">
         <v>1464</v>
       </c>
@@ -45085,7 +45085,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="559">
+    <row r="559" hidden="1">
       <c r="A559" s="3" t="s">
         <v>1466</v>
       </c>
@@ -45153,7 +45153,7 @@
       </c>
       <c r="W559" s="7"/>
     </row>
-    <row r="560">
+    <row r="560" hidden="1">
       <c r="A560" s="3" t="s">
         <v>1469</v>
       </c>
@@ -45221,7 +45221,7 @@
       </c>
       <c r="W560" s="7"/>
     </row>
-    <row r="561">
+    <row r="561" hidden="1">
       <c r="A561" s="3" t="s">
         <v>1469</v>
       </c>
@@ -45289,7 +45289,7 @@
       </c>
       <c r="W561" s="7"/>
     </row>
-    <row r="562">
+    <row r="562" hidden="1">
       <c r="A562" s="3" t="s">
         <v>1469</v>
       </c>
@@ -45357,7 +45357,7 @@
       </c>
       <c r="W562" s="7"/>
     </row>
-    <row r="563">
+    <row r="563" hidden="1">
       <c r="A563" s="3" t="s">
         <v>1469</v>
       </c>
@@ -45425,7 +45425,7 @@
       </c>
       <c r="W563" s="7"/>
     </row>
-    <row r="564">
+    <row r="564" hidden="1">
       <c r="A564" s="3" t="s">
         <v>1469</v>
       </c>
@@ -45493,7 +45493,7 @@
       </c>
       <c r="W564" s="7"/>
     </row>
-    <row r="565">
+    <row r="565" hidden="1">
       <c r="A565" s="3" t="s">
         <v>1480</v>
       </c>
@@ -45565,7 +45565,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="566">
+    <row r="566" hidden="1">
       <c r="A566" s="3" t="s">
         <v>1481</v>
       </c>
@@ -45703,7 +45703,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="568">
+    <row r="568" hidden="1">
       <c r="A568" s="3" t="s">
         <v>1486</v>
       </c>
@@ -45775,7 +45775,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="569">
+    <row r="569" hidden="1">
       <c r="A569" s="3" t="s">
         <v>1489</v>
       </c>
@@ -45913,7 +45913,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="571">
+    <row r="571" hidden="1">
       <c r="A571" s="3" t="s">
         <v>1495</v>
       </c>
@@ -45981,7 +45981,7 @@
       </c>
       <c r="W571" s="7"/>
     </row>
-    <row r="572">
+    <row r="572" hidden="1">
       <c r="A572" s="3" t="s">
         <v>1498</v>
       </c>
@@ -46053,7 +46053,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="573">
+    <row r="573" hidden="1">
       <c r="A573" s="3" t="s">
         <v>1501</v>
       </c>
@@ -46121,7 +46121,7 @@
       </c>
       <c r="W573" s="7"/>
     </row>
-    <row r="574">
+    <row r="574" hidden="1">
       <c r="A574" s="3" t="s">
         <v>1503</v>
       </c>
@@ -46193,7 +46193,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="575">
+    <row r="575" hidden="1">
       <c r="A575" s="3" t="s">
         <v>1506</v>
       </c>
@@ -46265,7 +46265,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="576">
+    <row r="576" hidden="1">
       <c r="A576" s="3" t="s">
         <v>1509</v>
       </c>
@@ -46337,7 +46337,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="577">
+    <row r="577" hidden="1">
       <c r="A577" s="3" t="s">
         <v>1512</v>
       </c>
@@ -46409,7 +46409,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="578">
+    <row r="578" hidden="1">
       <c r="A578" s="3" t="s">
         <v>1515</v>
       </c>
@@ -46481,7 +46481,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="579">
+    <row r="579" hidden="1">
       <c r="A579" s="3" t="s">
         <v>1518</v>
       </c>
@@ -46553,7 +46553,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="580">
+    <row r="580" hidden="1">
       <c r="A580" s="3" t="s">
         <v>1521</v>
       </c>
@@ -46621,7 +46621,7 @@
       </c>
       <c r="W580" s="7"/>
     </row>
-    <row r="581">
+    <row r="581" hidden="1">
       <c r="A581" s="3" t="s">
         <v>1524</v>
       </c>
@@ -46693,7 +46693,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="582">
+    <row r="582" hidden="1">
       <c r="A582" s="3" t="s">
         <v>1527</v>
       </c>
@@ -46835,7 +46835,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="584">
+    <row r="584" hidden="1">
       <c r="A584" s="3" t="s">
         <v>1532</v>
       </c>
@@ -46907,7 +46907,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="585">
+    <row r="585" hidden="1">
       <c r="A585" s="3" t="s">
         <v>1534</v>
       </c>
@@ -46975,7 +46975,7 @@
       </c>
       <c r="W585" s="7"/>
     </row>
-    <row r="586">
+    <row r="586" hidden="1">
       <c r="A586" s="3" t="s">
         <v>1537</v>
       </c>
@@ -47047,7 +47047,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="587">
+    <row r="587" hidden="1">
       <c r="A587" s="3" t="s">
         <v>1539</v>
       </c>
@@ -47119,7 +47119,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="588">
+    <row r="588" hidden="1">
       <c r="A588" s="3" t="s">
         <v>1542</v>
       </c>
@@ -47191,7 +47191,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="589">
+    <row r="589" hidden="1">
       <c r="A589" s="3" t="s">
         <v>1545</v>
       </c>
@@ -47263,7 +47263,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="590">
+    <row r="590" hidden="1">
       <c r="A590" s="3" t="s">
         <v>1548</v>
       </c>
@@ -47335,7 +47335,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="591">
+    <row r="591" hidden="1">
       <c r="A591" s="3" t="s">
         <v>1550</v>
       </c>
@@ -47407,7 +47407,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="592">
+    <row r="592" hidden="1">
       <c r="A592" s="3" t="s">
         <v>1553</v>
       </c>
@@ -47479,7 +47479,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="593">
+    <row r="593" hidden="1">
       <c r="A593" s="3" t="s">
         <v>1556</v>
       </c>
@@ -47551,7 +47551,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="594">
+    <row r="594" hidden="1">
       <c r="A594" s="3" t="s">
         <v>1556</v>
       </c>
@@ -47619,7 +47619,7 @@
       </c>
       <c r="W594" s="7"/>
     </row>
-    <row r="595">
+    <row r="595" hidden="1">
       <c r="A595" s="3" t="s">
         <v>1561</v>
       </c>
@@ -47691,7 +47691,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="596">
+    <row r="596" hidden="1">
       <c r="A596" s="3" t="s">
         <v>1563</v>
       </c>
@@ -47759,7 +47759,7 @@
       </c>
       <c r="W596" s="7"/>
     </row>
-    <row r="597">
+    <row r="597" hidden="1">
       <c r="A597" s="3" t="s">
         <v>1566</v>
       </c>
@@ -47831,7 +47831,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="598">
+    <row r="598" hidden="1">
       <c r="A598" s="3" t="s">
         <v>1569</v>
       </c>
@@ -47973,7 +47973,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="600">
+    <row r="600" hidden="1">
       <c r="A600" s="3" t="s">
         <v>1575</v>
       </c>
@@ -48115,7 +48115,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="602">
+    <row r="602" hidden="1">
       <c r="A602" s="3" t="s">
         <v>1580</v>
       </c>
@@ -48187,7 +48187,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="603">
+    <row r="603" hidden="1">
       <c r="A603" s="3" t="s">
         <v>1583</v>
       </c>
@@ -48259,7 +48259,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="604">
+    <row r="604" hidden="1">
       <c r="A604" s="3" t="s">
         <v>1585</v>
       </c>
@@ -48331,7 +48331,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="605">
+    <row r="605" hidden="1">
       <c r="A605" s="3" t="s">
         <v>1588</v>
       </c>
@@ -48399,7 +48399,7 @@
       </c>
       <c r="W605" s="7"/>
     </row>
-    <row r="606">
+    <row r="606" hidden="1">
       <c r="A606" s="3" t="s">
         <v>1591</v>
       </c>
@@ -48537,7 +48537,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="608">
+    <row r="608" hidden="1">
       <c r="A608" s="3" t="s">
         <v>1597</v>
       </c>
@@ -48609,7 +48609,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="609">
+    <row r="609" hidden="1">
       <c r="A609" s="3" t="s">
         <v>1600</v>
       </c>
@@ -48751,7 +48751,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="611">
+    <row r="611" hidden="1">
       <c r="A611" s="3" t="s">
         <v>1606</v>
       </c>
@@ -48819,7 +48819,7 @@
       </c>
       <c r="W611" s="3"/>
     </row>
-    <row r="612">
+    <row r="612" hidden="1">
       <c r="A612" s="3" t="s">
         <v>1608</v>
       </c>
@@ -48961,7 +48961,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="614">
+    <row r="614" hidden="1">
       <c r="A614" s="3" t="s">
         <v>1613</v>
       </c>
@@ -49033,7 +49033,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="615">
+    <row r="615" hidden="1">
       <c r="A615" s="3" t="s">
         <v>1616</v>
       </c>
@@ -49105,7 +49105,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="616">
+    <row r="616" hidden="1">
       <c r="A616" s="3" t="s">
         <v>1618</v>
       </c>
@@ -49177,7 +49177,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="617">
+    <row r="617" hidden="1">
       <c r="A617" s="3" t="s">
         <v>1621</v>
       </c>
@@ -49245,7 +49245,7 @@
       </c>
       <c r="W617" s="7"/>
     </row>
-    <row r="618">
+    <row r="618" hidden="1">
       <c r="A618" s="3" t="s">
         <v>1624</v>
       </c>
@@ -49313,7 +49313,7 @@
       </c>
       <c r="W618" s="7"/>
     </row>
-    <row r="619">
+    <row r="619" hidden="1">
       <c r="A619" s="3" t="s">
         <v>1627</v>
       </c>
@@ -49381,7 +49381,7 @@
       </c>
       <c r="W619" s="7"/>
     </row>
-    <row r="620">
+    <row r="620" hidden="1">
       <c r="A620" s="3" t="s">
         <v>1630</v>
       </c>
@@ -49453,7 +49453,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="621">
+    <row r="621" hidden="1">
       <c r="A621" s="3" t="s">
         <v>1632</v>
       </c>
@@ -49525,7 +49525,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="622">
+    <row r="622" hidden="1">
       <c r="A622" s="3" t="s">
         <v>1635</v>
       </c>
@@ -49593,7 +49593,7 @@
       </c>
       <c r="W622" s="7"/>
     </row>
-    <row r="623">
+    <row r="623" hidden="1">
       <c r="A623" s="3" t="s">
         <v>1638</v>
       </c>
@@ -49661,7 +49661,7 @@
       </c>
       <c r="W623" s="7"/>
     </row>
-    <row r="624">
+    <row r="624" hidden="1">
       <c r="A624" s="3" t="s">
         <v>1641</v>
       </c>
@@ -49731,7 +49731,7 @@
       </c>
       <c r="W624" s="3"/>
     </row>
-    <row r="625">
+    <row r="625" hidden="1">
       <c r="A625" s="3" t="s">
         <v>1644</v>
       </c>
@@ -49873,7 +49873,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="627">
+    <row r="627" hidden="1">
       <c r="A627" s="3" t="s">
         <v>1650</v>
       </c>
@@ -49945,7 +49945,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="628">
+    <row r="628" hidden="1">
       <c r="A628" s="3" t="s">
         <v>1653</v>
       </c>
@@ -50017,7 +50017,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="629">
+    <row r="629" hidden="1">
       <c r="A629" s="3" t="s">
         <v>1656</v>
       </c>
@@ -50089,7 +50089,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="630">
+    <row r="630" hidden="1">
       <c r="A630" s="3" t="s">
         <v>1659</v>
       </c>
@@ -50157,7 +50157,7 @@
       </c>
       <c r="W630" s="7"/>
     </row>
-    <row r="631">
+    <row r="631" hidden="1">
       <c r="A631" s="3" t="s">
         <v>1662</v>
       </c>
@@ -50299,7 +50299,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="633">
+    <row r="633" hidden="1">
       <c r="A633" s="3" t="s">
         <v>1667</v>
       </c>
@@ -50371,7 +50371,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="634">
+    <row r="634" hidden="1">
       <c r="A634" s="3" t="s">
         <v>1670</v>
       </c>
@@ -50444,7 +50444,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$AA$634"/>
+  <autoFilter ref="$A$1:$AA$634">
+    <filterColumn colId="21">
+      <filters blank="1">
+        <filter val="Not English"/>
+        <filter val="Not found"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink r:id="rId2" ref="B374"/>
     <hyperlink r:id="rId3" ref="B542"/>

</xml_diff>